<commit_message>
updated the data folder
</commit_message>
<xml_diff>
--- a/data/BladderCancer_trial_data_new.xlsx
+++ b/data/BladderCancer_trial_data_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/4476224/Desktop/RejniakLab_projects/Projects/Completed_2025_TIL_BC_proj/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/4476224/Desktop/RejniakLab_projects/Projects/2026_PETIL_proj/PETIL_70_30_spl/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8C8090B-01AB-4543-A27F-8E68414DEF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44DDCAB6-173E-7D40-9279-ED471B503CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="24460" windowHeight="13940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9680" yWindow="2080" windowWidth="24460" windowHeight="13940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="97">
   <si>
     <t>ID</t>
   </si>
@@ -322,9 +322,6 @@
   </si>
   <si>
     <t>HG Ta + CIS</t>
-  </si>
-  <si>
-    <t>Zemp</t>
   </si>
   <si>
     <t>Yes</t>
@@ -1827,28 +1824,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="8" customWidth="1"/>
     <col min="2" max="2" width="14.5" style="8" customWidth="1"/>
     <col min="3" max="3" width="15.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.83203125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="10.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.1640625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="10.5" style="8" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="15" style="9" customWidth="1"/>
-    <col min="12" max="12" width="23.83203125" style="8" customWidth="1"/>
-    <col min="13" max="13" width="21.5" style="8" customWidth="1"/>
-    <col min="14" max="14" width="23.83203125" style="8" customWidth="1"/>
-    <col min="15" max="15" width="18.1640625" style="8" customWidth="1"/>
-    <col min="16" max="16384" width="8.83203125" style="8"/>
+    <col min="4" max="4" width="12.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="10.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.1640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="10.5" style="8" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="15" style="9" customWidth="1"/>
+    <col min="11" max="11" width="23.83203125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="21.5" style="8" customWidth="1"/>
+    <col min="13" max="13" width="23.83203125" style="8" customWidth="1"/>
+    <col min="14" max="14" width="18.1640625" style="8" customWidth="1"/>
+    <col min="15" max="16384" width="8.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="3" customFormat="1" ht="81" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" s="3" customFormat="1" ht="81" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>83</v>
       </c>
@@ -1859,43 +1855,40 @@
         <v>93</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>9</v>
+        <v>73</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="O1" s="5" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>84</v>
       </c>
@@ -1906,39 +1899,36 @@
         <v>1158533</v>
       </c>
       <c r="D2" s="6">
+        <v>64</v>
+      </c>
+      <c r="E2" s="6">
+        <v>26.82</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6">
+        <v>1</v>
+      </c>
+      <c r="I2" s="6">
+        <v>2</v>
+      </c>
+      <c r="J2" s="6">
+        <v>0</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="L2" s="7"/>
+      <c r="M2" s="6">
         <v>7</v>
       </c>
-      <c r="E2" s="6">
-        <v>64</v>
-      </c>
-      <c r="F2" s="6">
-        <v>26.82</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6">
-        <v>1</v>
-      </c>
-      <c r="J2" s="6">
-        <v>2</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0.6</v>
-      </c>
-      <c r="M2" s="7"/>
-      <c r="N2" s="6">
-        <v>7</v>
-      </c>
-      <c r="O2" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N2" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>85</v>
       </c>
@@ -1949,39 +1939,36 @@
         <v>1154503</v>
       </c>
       <c r="D3" s="6">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="E3" s="6">
-        <v>73</v>
+        <v>23.81</v>
       </c>
       <c r="F3" s="6">
-        <v>23.81</v>
-      </c>
-      <c r="G3" s="6">
         <v>3</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6">
+        <v>1</v>
+      </c>
       <c r="I3" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" s="6">
         <v>2</v>
       </c>
       <c r="K3" s="6">
-        <v>2</v>
-      </c>
-      <c r="L3" s="6">
         <v>0.1</v>
       </c>
-      <c r="M3" s="7"/>
-      <c r="N3" s="6">
+      <c r="L3" s="7"/>
+      <c r="M3" s="6">
         <v>15</v>
       </c>
-      <c r="O3" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N3" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>86</v>
       </c>
@@ -1992,39 +1979,36 @@
         <v>1177617</v>
       </c>
       <c r="D4" s="6">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="E4" s="6">
-        <v>59</v>
+        <v>47.19</v>
       </c>
       <c r="F4" s="6">
-        <v>47.19</v>
-      </c>
-      <c r="G4" s="6">
         <v>1</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6">
+      <c r="G4" s="6"/>
+      <c r="H4" s="6">
         <v>1</v>
       </c>
-      <c r="J4" s="16">
+      <c r="I4" s="16">
         <v>2</v>
       </c>
+      <c r="J4" s="6">
+        <v>0</v>
+      </c>
       <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="M4" s="7"/>
-      <c r="N4" s="6">
+      <c r="L4" s="7"/>
+      <c r="M4" s="6">
         <v>48</v>
       </c>
-      <c r="O4" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N4" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>87</v>
       </c>
@@ -2035,39 +2019,36 @@
         <v>1154884</v>
       </c>
       <c r="D5" s="6">
+        <v>76</v>
+      </c>
+      <c r="E5" s="6">
+        <v>29.84</v>
+      </c>
+      <c r="F5" s="6">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6">
         <v>2</v>
       </c>
-      <c r="E5" s="6">
-        <v>76</v>
-      </c>
-      <c r="F5" s="6">
-        <v>29.84</v>
-      </c>
-      <c r="G5" s="6">
-        <v>1</v>
-      </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6">
-        <v>1</v>
-      </c>
       <c r="J5" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" s="6">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6">
         <v>0.2</v>
       </c>
-      <c r="M5" s="7"/>
-      <c r="N5" s="6">
+      <c r="L5" s="7"/>
+      <c r="M5" s="6">
         <v>7</v>
       </c>
-      <c r="O5" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N5" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>88</v>
       </c>
@@ -2078,39 +2059,36 @@
         <v>1207532</v>
       </c>
       <c r="D6" s="6">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="E6" s="6">
-        <v>77</v>
-      </c>
-      <c r="F6" s="6">
         <v>27.3</v>
       </c>
-      <c r="G6" s="16">
+      <c r="F6" s="16">
         <v>3</v>
       </c>
-      <c r="H6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6">
+        <v>1</v>
+      </c>
       <c r="I6" s="6">
+        <v>2</v>
+      </c>
+      <c r="J6" s="6">
         <v>1</v>
       </c>
-      <c r="J6" s="6">
-        <v>2</v>
-      </c>
       <c r="K6" s="6">
-        <v>1</v>
-      </c>
-      <c r="L6" s="6">
         <v>1.4</v>
       </c>
-      <c r="M6" s="7"/>
-      <c r="N6" s="6">
+      <c r="L6" s="7"/>
+      <c r="M6" s="6">
         <v>35</v>
       </c>
-      <c r="O6" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N6" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>89</v>
       </c>
@@ -2121,39 +2099,36 @@
         <v>1234800</v>
       </c>
       <c r="D7" s="6">
+        <v>77</v>
+      </c>
+      <c r="E7" s="6">
+        <v>26.45</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6">
         <v>1</v>
       </c>
-      <c r="E7" s="6">
-        <v>77</v>
-      </c>
-      <c r="F7" s="6">
-        <v>26.45</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="H7" s="6"/>
       <c r="I7" s="6">
+        <v>2</v>
+      </c>
+      <c r="J7" s="6">
         <v>1</v>
       </c>
-      <c r="J7" s="6">
-        <v>2</v>
-      </c>
       <c r="K7" s="6">
-        <v>1</v>
-      </c>
-      <c r="L7" s="6">
         <v>0.5</v>
       </c>
-      <c r="M7" s="7"/>
-      <c r="N7" s="6">
+      <c r="L7" s="7"/>
+      <c r="M7" s="6">
         <v>28</v>
       </c>
-      <c r="O7" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N7" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>90</v>
       </c>
@@ -2163,40 +2138,37 @@
       <c r="C8" s="13">
         <v>1160124</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="6">
+        <v>84</v>
+      </c>
+      <c r="E8" s="6">
+        <v>25.54</v>
+      </c>
+      <c r="F8" s="16">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6">
+        <v>2</v>
+      </c>
+      <c r="J8" s="6">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="L8" s="7"/>
+      <c r="M8" s="6">
+        <v>14</v>
+      </c>
+      <c r="N8" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="6">
-        <v>84</v>
-      </c>
-      <c r="F8" s="6">
-        <v>25.54</v>
-      </c>
-      <c r="G8" s="16">
-        <v>1</v>
-      </c>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6">
-        <v>1</v>
-      </c>
-      <c r="J8" s="6">
-        <v>2</v>
-      </c>
-      <c r="K8" s="6">
-        <v>0</v>
-      </c>
-      <c r="L8" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="6">
-        <v>14</v>
-      </c>
-      <c r="O8" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>91</v>
       </c>
@@ -2206,40 +2178,37 @@
       <c r="C9" s="13">
         <v>1247334</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="6">
+        <v>69</v>
+      </c>
+      <c r="E9" s="6">
+        <v>28.12</v>
+      </c>
+      <c r="F9" s="16">
+        <v>2</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6">
+        <v>2</v>
+      </c>
+      <c r="J9" s="6">
+        <v>1</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="L9" s="7"/>
+      <c r="M9" s="6">
+        <v>6</v>
+      </c>
+      <c r="N9" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="E9" s="6">
-        <v>69</v>
-      </c>
-      <c r="F9" s="6">
-        <v>28.12</v>
-      </c>
-      <c r="G9" s="16">
-        <v>2</v>
-      </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6">
-        <v>2</v>
-      </c>
-      <c r="K9" s="6">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="6">
-        <v>6</v>
-      </c>
-      <c r="O9" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>92</v>
       </c>
@@ -2250,46 +2219,42 @@
         <v>1199367</v>
       </c>
       <c r="D10" s="6">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="E10" s="6">
-        <v>64</v>
+        <v>27.95</v>
       </c>
       <c r="F10" s="6">
-        <v>27.95</v>
-      </c>
-      <c r="G10" s="6">
         <v>1</v>
       </c>
-      <c r="H10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6">
+        <v>1</v>
+      </c>
       <c r="I10" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" s="6">
-        <v>0</v>
-      </c>
-      <c r="L10" s="6">
         <v>0.2</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="6">
+      <c r="L10" s="7"/>
+      <c r="M10" s="6">
         <v>13</v>
       </c>
-      <c r="O10" s="12" t="s">
-        <v>97</v>
+      <c r="N10" s="12" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations xWindow="938" yWindow="226" count="6">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0-T0 7-T3_x000a_1-Ta 8-T3a_x000a_2-Tis 9-T3b_x000a_3-T1 10-T4_x000a_4-T2 11-T4a_x000a_5-T2a 12-T4b_x000a_6-T2b 13-Tx_x000a_" sqref="G1" xr:uid="{00000000-0002-0000-0000-00001C000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 - Unknown/Other_x000a_1 - White_x000a_2 - Black_x000a_3 - Asian_x000a_4 - Naïve Hawaiian/Pacific Islander_x000a_5 - American Indian/Alaskan Native" sqref="I1" xr:uid="{00000000-0002-0000-0000-000021000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="1 = Sexton   5 = Gilbert_x000a_2 = Spiess   6 = Manley_x000a_3 = PowSang  7 = Li_x000a_4 = Poch_x000a_" sqref="D1" xr:uid="{00000000-0002-0000-0000-000023000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 = T0     8 = T3a_x000a_1 = Ta      9 = T3b_x000a_2 = Tis      10 = T4_x000a_3 = T1      11 = T4a_x000a_4 = T2      12 = T4b_x000a_5 = T2a     13 = TX_x000a_6 = T2b     _x000a_7 = T3" sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0000-000016000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="1 = Radical Cystectomy_x000a_2 = TURBT" sqref="J1:J1048576" xr:uid="{CD3F280F-85D1-254C-8AE5-90AE82D0BCEE}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 - Never Smoked_x000a_1 - Ever Smoked_x000a_2 - Current Smoker" sqref="K1:K1048576" xr:uid="{474D1087-1F4A-BA41-932B-9F2F0228F032}"/>
+  <dataValidations xWindow="938" yWindow="226" count="5">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0-T0 7-T3_x000a_1-Ta 8-T3a_x000a_2-Tis 9-T3b_x000a_3-T1 10-T4_x000a_4-T2 11-T4a_x000a_5-T2a 12-T4b_x000a_6-T2b 13-Tx_x000a_" sqref="F1" xr:uid="{00000000-0002-0000-0000-00001C000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 - Unknown/Other_x000a_1 - White_x000a_2 - Black_x000a_3 - Asian_x000a_4 - Naïve Hawaiian/Pacific Islander_x000a_5 - American Indian/Alaskan Native" sqref="H1" xr:uid="{00000000-0002-0000-0000-000021000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 = T0     8 = T3a_x000a_1 = Ta      9 = T3b_x000a_2 = Tis      10 = T4_x000a_3 = T1      11 = T4a_x000a_4 = T2      12 = T4b_x000a_5 = T2a     13 = TX_x000a_6 = T2b     _x000a_7 = T3" sqref="G1:G1048576" xr:uid="{00000000-0002-0000-0000-000016000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="1 = Radical Cystectomy_x000a_2 = TURBT" sqref="I1:I1048576" xr:uid="{CD3F280F-85D1-254C-8AE5-90AE82D0BCEE}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="0 - Never Smoked_x000a_1 - Ever Smoked_x000a_2 - Current Smoker" sqref="J1:J1048576" xr:uid="{474D1087-1F4A-BA41-932B-9F2F0228F032}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>